<commit_message>
Finalize verified W2 lineup (401 rows) + timetable docs
</commit_message>
<xml_diff>
--- a/Tomorrowland_2026_W2_timetable.xlsx
+++ b/Tomorrowland_2026_W2_timetable.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D142"/>
+  <dimension ref="A1:D141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1642,22 +1642,22 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>ELIXIR</t>
+          <t>FREEDOM BY BUD</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>01:00</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>Hide N Seek</t>
+          <t>Esin Boz</t>
         </is>
       </c>
     </row>
@@ -1669,17 +1669,17 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Esin Boz</t>
+          <t>JOA</t>
         </is>
       </c>
     </row>
@@ -1691,17 +1691,17 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>JOA</t>
+          <t>Aaron Hibell</t>
         </is>
       </c>
     </row>
@@ -1713,17 +1713,17 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>Aaron Hibell</t>
+          <t>Amber Broos b2b Juliet Fox</t>
         </is>
       </c>
     </row>
@@ -1735,17 +1735,17 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>17:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>Amber Broos b2b Juliet Fox</t>
+          <t>Enrico Sangiuliano</t>
         </is>
       </c>
     </row>
@@ -1757,17 +1757,17 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>17:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Enrico Sangiuliano</t>
+          <t>John Newman (Live band)</t>
         </is>
       </c>
     </row>
@@ -1779,17 +1779,17 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>John Newman (Live band)</t>
+          <t>Bebe Rexha</t>
         </is>
       </c>
     </row>
@@ -1801,17 +1801,17 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Bebe Rexha</t>
+          <t>James Hype</t>
         </is>
       </c>
     </row>
@@ -1823,17 +1823,17 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>James Hype</t>
+          <t>Fisher</t>
         </is>
       </c>
     </row>
@@ -1845,39 +1845,39 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>00:30</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Fisher</t>
+          <t>Alesso</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>FREEDOM BY BUD</t>
+          <t>HOUSE OF FORTUNE BY JBL</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>00:30</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>Alesso</t>
+          <t>Reygel</t>
         </is>
       </c>
     </row>
@@ -1889,17 +1889,17 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Reygel</t>
+          <t>Alan Alvarez &amp; CRAZY SIR-G</t>
         </is>
       </c>
     </row>
@@ -1911,17 +1911,17 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>Alan Alvarez &amp; CRAZY SIR-G</t>
+          <t>Martin Trevy</t>
         </is>
       </c>
     </row>
@@ -1933,17 +1933,17 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Martin Trevy</t>
+          <t>Vinne</t>
         </is>
       </c>
     </row>
@@ -1955,17 +1955,17 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>Vinne</t>
+          <t>Ely Oaks</t>
         </is>
       </c>
     </row>
@@ -1977,17 +1977,17 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>Ely Oaks</t>
+          <t>ELFIGO</t>
         </is>
       </c>
     </row>
@@ -1999,17 +1999,17 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>ELFIGO</t>
+          <t>Telykast</t>
         </is>
       </c>
     </row>
@@ -2021,17 +2021,17 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>Telykast</t>
+          <t>Didi Han</t>
         </is>
       </c>
     </row>
@@ -2043,39 +2043,39 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>Didi Han</t>
+          <t>MEGURU</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>HOUSE OF FORTUNE BY JBL</t>
+          <t>MAINSTAGE</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>MEGURU</t>
+          <t>DISCOVERY</t>
         </is>
       </c>
     </row>
@@ -2087,17 +2087,17 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>DISCOVERY</t>
+          <t>More to be announced</t>
         </is>
       </c>
     </row>
@@ -2109,17 +2109,17 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>More to be announced</t>
+          <t>Ely Oaks</t>
         </is>
       </c>
     </row>
@@ -2131,17 +2131,17 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>Ely Oaks</t>
+          <t>Yves V</t>
         </is>
       </c>
     </row>
@@ -2153,17 +2153,17 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>17:30</t>
+          <t>18:35</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>Yves V</t>
+          <t>Miss Monique</t>
         </is>
       </c>
     </row>
@@ -2175,17 +2175,17 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>18:40</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>18:35</t>
+          <t>19:40</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>Miss Monique</t>
+          <t>Indira Paganotto</t>
         </is>
       </c>
     </row>
@@ -2197,17 +2197,17 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>18:40</t>
+          <t>19:40</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>19:40</t>
+          <t>20:40</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>Indira Paganotto</t>
+          <t>Nicky Romero</t>
         </is>
       </c>
     </row>
@@ -2219,17 +2219,17 @@
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>19:40</t>
+          <t>20:40</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>20:40</t>
+          <t>21:40</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>Nicky Romero</t>
+          <t>Kölsch</t>
         </is>
       </c>
     </row>
@@ -2241,17 +2241,17 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>20:40</t>
+          <t>21:45</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>21:40</t>
+          <t>22:45</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>Kölsch</t>
+          <t>Alok</t>
         </is>
       </c>
     </row>
@@ -2263,17 +2263,17 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>21:45</t>
+          <t>22:50</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>22:45</t>
+          <t>23:50</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>Alok</t>
+          <t>Steve Angello</t>
         </is>
       </c>
     </row>
@@ -2285,39 +2285,39 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>22:50</t>
+          <t>23:50</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>23:50</t>
+          <t>00:50</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>Steve Angello</t>
+          <t>Hardwell</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>MAINSTAGE</t>
+          <t>MELODIA BY CORONA</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>23:50</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>00:50</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>Hardwell</t>
+          <t>SPIES</t>
         </is>
       </c>
     </row>
@@ -2329,17 +2329,17 @@
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>SPIES</t>
+          <t>Joulie</t>
         </is>
       </c>
     </row>
@@ -2351,17 +2351,17 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>Joulie</t>
+          <t>L-Fêtes</t>
         </is>
       </c>
     </row>
@@ -2373,17 +2373,17 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>19:15</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>L-Fêtes</t>
+          <t>Planet Groove DJ's</t>
         </is>
       </c>
     </row>
@@ -2395,17 +2395,17 @@
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>19:15</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>19:15</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>Planet Groove DJ's</t>
+          <t>Eko Roosevelt Live</t>
         </is>
       </c>
     </row>
@@ -2417,17 +2417,17 @@
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>19:15</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>Eko Roosevelt Live</t>
+          <t>John Noseda</t>
         </is>
       </c>
     </row>
@@ -2439,39 +2439,39 @@
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>John Noseda</t>
+          <t>Jeroen Delodder</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>MELODIA BY CORONA</t>
+          <t>MOOSE BAR</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>Jeroen Delodder</t>
+          <t>Prosit</t>
         </is>
       </c>
     </row>
@@ -2483,17 +2483,17 @@
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>Prosit</t>
+          <t>Jo Cox</t>
         </is>
       </c>
     </row>
@@ -2505,17 +2505,17 @@
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>Jo Cox</t>
+          <t>Otto Wunderbar</t>
         </is>
       </c>
     </row>
@@ -2527,39 +2527,39 @@
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>Otto Wunderbar</t>
+          <t>The Bobmeister</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>MOOSE BAR</t>
+          <t>PLANAXIS</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>The Bobmeister</t>
+          <t>Locus</t>
         </is>
       </c>
     </row>
@@ -2571,17 +2571,17 @@
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>Locus</t>
+          <t>Domi Re</t>
         </is>
       </c>
     </row>
@@ -2593,17 +2593,17 @@
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>Domi Re</t>
+          <t>Beat Controllers</t>
         </is>
       </c>
     </row>
@@ -2615,17 +2615,17 @@
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>Beat Controllers</t>
+          <t>Vitor Falabella</t>
         </is>
       </c>
     </row>
@@ -2637,17 +2637,17 @@
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>Vitor Falabella</t>
+          <t>Firaga</t>
         </is>
       </c>
     </row>
@@ -2659,17 +2659,17 @@
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>Firaga</t>
+          <t>Somnia</t>
         </is>
       </c>
     </row>
@@ -2681,17 +2681,17 @@
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>Somnia</t>
+          <t>Phaxe</t>
         </is>
       </c>
     </row>
@@ -2703,17 +2703,17 @@
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="D103" s="2" t="inlineStr">
         <is>
-          <t>Phaxe</t>
+          <t>Blazy</t>
         </is>
       </c>
     </row>
@@ -2725,17 +2725,17 @@
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>Blazy</t>
+          <t>Blastoyz</t>
         </is>
       </c>
     </row>
@@ -2747,17 +2747,17 @@
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
         <is>
-          <t>Blastoyz</t>
+          <t>Vegas</t>
         </is>
       </c>
     </row>
@@ -2769,17 +2769,17 @@
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>Vegas</t>
+          <t>Avalon</t>
         </is>
       </c>
     </row>
@@ -2791,39 +2791,39 @@
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr">
         <is>
-          <t>Avalon</t>
+          <t>Electric Universe</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>PLANAXIS</t>
+          <t>THE GREAT LIBRARY</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
-          <t>Electric Universe</t>
+          <t>Calumny</t>
         </is>
       </c>
     </row>
@@ -2835,17 +2835,17 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="D109" s="2" t="inlineStr">
         <is>
-          <t>Calumny</t>
+          <t>Meaghan</t>
         </is>
       </c>
     </row>
@@ -2857,17 +2857,17 @@
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
-          <t>Meaghan</t>
+          <t>NOME.</t>
         </is>
       </c>
     </row>
@@ -2879,17 +2879,17 @@
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="D111" s="2" t="inlineStr">
         <is>
-          <t>NOME.</t>
+          <t>5NAPBACK</t>
         </is>
       </c>
     </row>
@@ -2901,17 +2901,17 @@
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="D112" s="2" t="inlineStr">
         <is>
-          <t>5NAPBACK</t>
+          <t>Merow</t>
         </is>
       </c>
     </row>
@@ -2923,17 +2923,17 @@
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="D113" s="2" t="inlineStr">
         <is>
-          <t>Merow</t>
+          <t>B Jones</t>
         </is>
       </c>
     </row>
@@ -2945,17 +2945,17 @@
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="D114" s="2" t="inlineStr">
         <is>
-          <t>B Jones</t>
+          <t>Regi</t>
         </is>
       </c>
     </row>
@@ -2967,17 +2967,17 @@
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="C115" s="2" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="D115" s="2" t="inlineStr">
         <is>
-          <t>Regi</t>
+          <t>MANDY</t>
         </is>
       </c>
     </row>
@@ -2989,17 +2989,17 @@
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="D116" s="2" t="inlineStr">
         <is>
-          <t>MANDY</t>
+          <t>Omdat Het Kan &amp; Average Rob</t>
         </is>
       </c>
     </row>
@@ -3011,17 +3011,17 @@
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="D117" s="2" t="inlineStr">
         <is>
-          <t>Omdat Het Kan &amp; Average Rob</t>
+          <t>HALŌ</t>
         </is>
       </c>
     </row>
@@ -3033,17 +3033,17 @@
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="D118" s="2" t="inlineStr">
         <is>
-          <t>HALŌ</t>
+          <t>Kaskade</t>
         </is>
       </c>
     </row>
@@ -3055,17 +3055,17 @@
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="C119" s="2" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="D119" s="2" t="inlineStr">
         <is>
-          <t>Kaskade</t>
+          <t>Alan Walker</t>
         </is>
       </c>
     </row>
@@ -3077,39 +3077,39 @@
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:55</t>
         </is>
       </c>
       <c r="D120" s="2" t="inlineStr">
         <is>
-          <t>Alan Walker</t>
+          <t>Illenium</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>THE GREAT LIBRARY</t>
+          <t>THE RAVE CAVE</t>
         </is>
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="C121" s="2" t="inlineStr">
         <is>
-          <t>00:55</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="D121" s="2" t="inlineStr">
         <is>
-          <t>Illenium</t>
+          <t>Sanne Dammers</t>
         </is>
       </c>
     </row>
@@ -3121,17 +3121,17 @@
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="C122" s="2" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="D122" s="2" t="inlineStr">
         <is>
-          <t>Sanne Dammers</t>
+          <t>Leesa</t>
         </is>
       </c>
     </row>
@@ -3143,17 +3143,17 @@
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="C123" s="2" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="D123" s="2" t="inlineStr">
         <is>
-          <t>Leesa</t>
+          <t>VIKTÖR b2b MZDZ</t>
         </is>
       </c>
     </row>
@@ -3165,17 +3165,17 @@
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="C124" s="2" t="inlineStr">
         <is>
-          <t>17:30</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="D124" s="2" t="inlineStr">
         <is>
-          <t>VIKTÖR b2b MZDZ</t>
+          <t>Lou8</t>
         </is>
       </c>
     </row>
@@ -3187,17 +3187,17 @@
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
-          <t>17:30</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="C125" s="2" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="D125" s="2" t="inlineStr">
         <is>
-          <t>Lou8</t>
+          <t>Jared</t>
         </is>
       </c>
     </row>
@@ -3209,17 +3209,17 @@
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="C126" s="2" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="D126" s="2" t="inlineStr">
         <is>
-          <t>Jared</t>
+          <t>Xijaro &amp; Pitch</t>
         </is>
       </c>
     </row>
@@ -3231,17 +3231,17 @@
       </c>
       <c r="B127" s="2" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="C127" s="2" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="D127" s="2" t="inlineStr">
         <is>
-          <t>Xijaro &amp; Pitch</t>
+          <t>Mr. Joy</t>
         </is>
       </c>
     </row>
@@ -3253,17 +3253,17 @@
       </c>
       <c r="B128" s="2" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="C128" s="2" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="D128" s="2" t="inlineStr">
         <is>
-          <t>Mr. Joy</t>
+          <t>Mairee</t>
         </is>
       </c>
     </row>
@@ -3275,39 +3275,39 @@
       </c>
       <c r="B129" s="2" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="C129" s="2" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="D129" s="2" t="inlineStr">
         <is>
-          <t>Mairee</t>
+          <t>Bisoux b2b Jef Nice</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>THE RAVE CAVE</t>
+          <t>THE ROSE GARDEN</t>
         </is>
       </c>
       <c r="B130" s="2" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="C130" s="2" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="D130" s="2" t="inlineStr">
         <is>
-          <t>Bisoux b2b Jef Nice</t>
+          <t>Shawiya Tribe</t>
         </is>
       </c>
     </row>
@@ -3319,17 +3319,17 @@
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="C131" s="2" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="D131" s="2" t="inlineStr">
         <is>
-          <t>Shawiya Tribe</t>
+          <t>LICIA</t>
         </is>
       </c>
     </row>
@@ -3341,17 +3341,17 @@
       </c>
       <c r="B132" s="2" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="C132" s="2" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="D132" s="2" t="inlineStr">
         <is>
-          <t>LICIA</t>
+          <t>Lucky Luke</t>
         </is>
       </c>
     </row>
@@ -3363,17 +3363,17 @@
       </c>
       <c r="B133" s="2" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="C133" s="2" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="D133" s="2" t="inlineStr">
         <is>
-          <t>Lucky Luke</t>
+          <t>Goddard &amp; Dread MC</t>
         </is>
       </c>
     </row>
@@ -3385,17 +3385,17 @@
       </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C134" s="2" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="D134" s="2" t="inlineStr">
         <is>
-          <t>Goddard &amp; Dread MC</t>
+          <t>Ghengar</t>
         </is>
       </c>
     </row>
@@ -3407,17 +3407,17 @@
       </c>
       <c r="B135" s="2" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="C135" s="2" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="D135" s="2" t="inlineStr">
         <is>
-          <t>Ghengar</t>
+          <t>ALLEYCVT</t>
         </is>
       </c>
     </row>
@@ -3429,17 +3429,17 @@
       </c>
       <c r="B136" s="2" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="C136" s="2" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="D136" s="2" t="inlineStr">
         <is>
-          <t>ALLEYCVT</t>
+          <t>Basstripper</t>
         </is>
       </c>
     </row>
@@ -3451,17 +3451,17 @@
       </c>
       <c r="B137" s="2" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="C137" s="2" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="D137" s="2" t="inlineStr">
         <is>
-          <t>Basstripper</t>
+          <t>Jessica Audiffred</t>
         </is>
       </c>
     </row>
@@ -3473,17 +3473,17 @@
       </c>
       <c r="B138" s="2" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="C138" s="2" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="D138" s="2" t="inlineStr">
         <is>
-          <t>Jessica Audiffred</t>
+          <t>Riot Ten</t>
         </is>
       </c>
     </row>
@@ -3495,17 +3495,17 @@
       </c>
       <c r="B139" s="2" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="C139" s="2" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="D139" s="2" t="inlineStr">
         <is>
-          <t>Riot Ten</t>
+          <t>BOU + B LIVE 247</t>
         </is>
       </c>
     </row>
@@ -3517,17 +3517,17 @@
       </c>
       <c r="B140" s="2" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="C140" s="2" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="D140" s="2" t="inlineStr">
         <is>
-          <t>BOU + B LIVE 247</t>
+          <t>Borgore</t>
         </is>
       </c>
     </row>
@@ -3539,37 +3539,15 @@
       </c>
       <c r="B141" s="2" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="C141" s="2" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>01:00</t>
         </is>
       </c>
       <c r="D141" s="2" t="inlineStr">
-        <is>
-          <t>Borgore</t>
-        </is>
-      </c>
-    </row>
-    <row r="142">
-      <c r="A142" s="2" t="inlineStr">
-        <is>
-          <t>THE ROSE GARDEN</t>
-        </is>
-      </c>
-      <c r="B142" s="2" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="C142" s="2" t="inlineStr">
-        <is>
-          <t>01:00</t>
-        </is>
-      </c>
-      <c r="D142" s="2" t="inlineStr">
         <is>
           <t>Sullivan King</t>
         </is>
@@ -3586,7 +3564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D133"/>
+  <dimension ref="A1:D134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -4945,17 +4923,17 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
           <t>22:00</t>
         </is>
       </c>
-      <c r="C62" s="2" t="inlineStr">
-        <is>
-          <t>23:00</t>
-        </is>
-      </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Sebastian Ingrosso</t>
+          <t>Symphony Of Unity</t>
         </is>
       </c>
     </row>
@@ -4967,39 +4945,39 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
           <t>23:00</t>
         </is>
       </c>
-      <c r="C63" s="2" t="inlineStr">
-        <is>
-          <t>00:30</t>
-        </is>
-      </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>Timmy Trumpet</t>
+          <t>Sebastian Ingrosso</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>HOUSE OF FORTUNE BY JBL</t>
+          <t>FREEDOM BY BUD</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>00:30</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Triciaa</t>
+          <t>Timmy Trumpet</t>
         </is>
       </c>
     </row>
@@ -5011,17 +4989,17 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
           <t>14:00</t>
         </is>
       </c>
-      <c r="C65" s="2" t="inlineStr">
-        <is>
-          <t>14:30</t>
-        </is>
-      </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>Likki</t>
+          <t>Triciaa</t>
         </is>
       </c>
     </row>
@@ -5033,17 +5011,17 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
           <t>14:30</t>
         </is>
       </c>
-      <c r="C66" s="2" t="inlineStr">
-        <is>
-          <t>15:00</t>
-        </is>
-      </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Gaddi</t>
+          <t>Likki</t>
         </is>
       </c>
     </row>
@@ -5055,17 +5033,17 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
           <t>15:00</t>
         </is>
       </c>
-      <c r="C67" s="2" t="inlineStr">
-        <is>
-          <t>15:30</t>
-        </is>
-      </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>Rassix</t>
+          <t>Gaddi</t>
         </is>
       </c>
     </row>
@@ -5077,17 +5055,17 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
           <t>15:30</t>
         </is>
       </c>
-      <c r="C68" s="2" t="inlineStr">
-        <is>
-          <t>16:00</t>
-        </is>
-      </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>TOO BIASED</t>
+          <t>Rassix</t>
         </is>
       </c>
     </row>
@@ -5099,17 +5077,17 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
           <t>16:00</t>
         </is>
       </c>
-      <c r="C69" s="2" t="inlineStr">
-        <is>
-          <t>17:00</t>
-        </is>
-      </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>Yaz.</t>
+          <t>TOO BIASED</t>
         </is>
       </c>
     </row>
@@ -5121,17 +5099,17 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
           <t>17:00</t>
         </is>
       </c>
-      <c r="C70" s="2" t="inlineStr">
-        <is>
-          <t>18:00</t>
-        </is>
-      </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>Carly Wilford</t>
+          <t>Yaz.</t>
         </is>
       </c>
     </row>
@@ -5143,17 +5121,17 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
           <t>18:00</t>
         </is>
       </c>
-      <c r="C71" s="2" t="inlineStr">
-        <is>
-          <t>19:00</t>
-        </is>
-      </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>Mosimann</t>
+          <t>Carly Wilford</t>
         </is>
       </c>
     </row>
@@ -5165,17 +5143,17 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
           <t>19:00</t>
         </is>
       </c>
-      <c r="C72" s="2" t="inlineStr">
-        <is>
-          <t>20:00</t>
-        </is>
-      </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>Nosefin</t>
+          <t>Mosimann</t>
         </is>
       </c>
     </row>
@@ -5187,17 +5165,17 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
           <t>20:00</t>
         </is>
       </c>
-      <c r="C73" s="2" t="inlineStr">
-        <is>
-          <t>21:00</t>
-        </is>
-      </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>More to be announced</t>
+          <t>Nosefin</t>
         </is>
       </c>
     </row>
@@ -5209,39 +5187,39 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
           <t>21:00</t>
         </is>
       </c>
-      <c r="C74" s="2" t="inlineStr">
-        <is>
-          <t>22:00</t>
-        </is>
-      </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>Atkö</t>
+          <t>More to be announced</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>MAINSTAGE</t>
+          <t>HOUSE OF FORTUNE BY JBL</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>DISCOVERY</t>
+          <t>Atkö</t>
         </is>
       </c>
     </row>
@@ -5253,17 +5231,17 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
           <t>14:00</t>
         </is>
       </c>
-      <c r="C76" s="2" t="inlineStr">
-        <is>
-          <t>15:00</t>
-        </is>
-      </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>Angemi</t>
+          <t>DISCOVERY</t>
         </is>
       </c>
     </row>
@@ -5275,17 +5253,17 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
           <t>15:00</t>
         </is>
       </c>
-      <c r="C77" s="2" t="inlineStr">
-        <is>
-          <t>16:15</t>
-        </is>
-      </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>Mike Williams</t>
+          <t>Angemi</t>
         </is>
       </c>
     </row>
@@ -5297,17 +5275,17 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
           <t>16:15</t>
         </is>
       </c>
-      <c r="C78" s="2" t="inlineStr">
-        <is>
-          <t>17:15</t>
-        </is>
-      </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>D.O.D</t>
+          <t>Mike Williams</t>
         </is>
       </c>
     </row>
@@ -5319,17 +5297,17 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>17:20</t>
+          <t>16:15</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>18:20</t>
+          <t>17:15</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>MATTN</t>
+          <t>D.O.D</t>
         </is>
       </c>
     </row>
@@ -5341,17 +5319,17 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
+          <t>17:20</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
           <t>18:20</t>
         </is>
       </c>
-      <c r="C80" s="2" t="inlineStr">
-        <is>
-          <t>19:20</t>
-        </is>
-      </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>Morten</t>
+          <t>MATTN</t>
         </is>
       </c>
     </row>
@@ -5363,17 +5341,17 @@
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
+          <t>18:20</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
           <t>19:20</t>
         </is>
       </c>
-      <c r="C81" s="2" t="inlineStr">
-        <is>
-          <t>20:20</t>
-        </is>
-      </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>Agents of Time</t>
+          <t>Morten</t>
         </is>
       </c>
     </row>
@@ -5385,17 +5363,17 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>20:25</t>
+          <t>19:20</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>21:25</t>
+          <t>20:20</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>Sub Zero Project</t>
+          <t>Agents of Time</t>
         </is>
       </c>
     </row>
@@ -5407,17 +5385,17 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
+          <t>20:25</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
           <t>21:25</t>
         </is>
       </c>
-      <c r="C83" s="2" t="inlineStr">
-        <is>
-          <t>22:25</t>
-        </is>
-      </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>Armin van Buuren</t>
+          <t>Sub Zero Project</t>
         </is>
       </c>
     </row>
@@ -5429,17 +5407,17 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>22:30</t>
+          <t>21:25</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>23:45</t>
+          <t>22:25</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>Dimitri Vegas &amp; Like Mike</t>
+          <t>Armin van Buuren</t>
         </is>
       </c>
     </row>
@@ -5451,39 +5429,39 @@
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
+          <t>22:30</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
           <t>23:45</t>
         </is>
       </c>
-      <c r="C85" s="2" t="inlineStr">
-        <is>
-          <t>00:45</t>
-        </is>
-      </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>Calvin Harris</t>
+          <t>Dimitri Vegas &amp; Like Mike</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>MELODIA BY CORONA</t>
+          <t>MAINSTAGE</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>23:45</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>00:45</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>Mooris</t>
+          <t>Calvin Harris</t>
         </is>
       </c>
     </row>
@@ -5495,17 +5473,17 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
           <t>14:00</t>
         </is>
       </c>
-      <c r="C87" s="2" t="inlineStr">
-        <is>
-          <t>15:30</t>
-        </is>
-      </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>Emilia De La Paz</t>
+          <t>Mooris</t>
         </is>
       </c>
     </row>
@@ -5517,17 +5495,17 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
           <t>15:30</t>
         </is>
       </c>
-      <c r="C88" s="2" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>Soulastico b2b Tohma</t>
+          <t>Emilia De La Paz</t>
         </is>
       </c>
     </row>
@@ -5539,17 +5517,17 @@
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
           <t>17:30</t>
         </is>
       </c>
-      <c r="C89" s="2" t="inlineStr">
-        <is>
-          <t>19:00</t>
-        </is>
-      </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>Larry Masmero</t>
+          <t>Soulastico b2b Tohma</t>
         </is>
       </c>
     </row>
@@ -5561,17 +5539,17 @@
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
           <t>19:00</t>
         </is>
       </c>
-      <c r="C90" s="2" t="inlineStr">
-        <is>
-          <t>20:30</t>
-        </is>
-      </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>Geheimzinnig Soundsystem</t>
+          <t>Larry Masmero</t>
         </is>
       </c>
     </row>
@@ -5583,17 +5561,17 @@
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
           <t>20:30</t>
         </is>
       </c>
-      <c r="C91" s="2" t="inlineStr">
-        <is>
-          <t>22:00</t>
-        </is>
-      </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>Séa</t>
+          <t>Geheimzinnig Soundsystem</t>
         </is>
       </c>
     </row>
@@ -5605,39 +5583,39 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
           <t>22:00</t>
         </is>
       </c>
-      <c r="C92" s="2" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>Sam Girling</t>
+          <t>Séa</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>MOOSE BAR</t>
+          <t>MELODIA BY CORONA</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>Mobius One</t>
+          <t>Sam Girling</t>
         </is>
       </c>
     </row>
@@ -5649,17 +5627,17 @@
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
           <t>15:00</t>
         </is>
       </c>
-      <c r="C94" s="2" t="inlineStr">
-        <is>
-          <t>19:00</t>
-        </is>
-      </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>Mr. E</t>
+          <t>Mobius One</t>
         </is>
       </c>
     </row>
@@ -5671,17 +5649,17 @@
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
           <t>19:00</t>
         </is>
       </c>
-      <c r="C95" s="2" t="inlineStr">
-        <is>
-          <t>20:00</t>
-        </is>
-      </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>De Romeo's</t>
+          <t>Mr. E</t>
         </is>
       </c>
     </row>
@@ -5693,39 +5671,39 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
           <t>20:00</t>
         </is>
       </c>
-      <c r="C96" s="2" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>Kurt Verheyen</t>
+          <t>De Romeo's</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>PLANAXIS</t>
+          <t>MOOSE BAR</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>NA:TUS</t>
+          <t>Kurt Verheyen</t>
         </is>
       </c>
     </row>
@@ -5737,17 +5715,17 @@
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
           <t>13:30</t>
         </is>
       </c>
-      <c r="C98" s="2" t="inlineStr">
-        <is>
-          <t>15:00</t>
-        </is>
-      </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>Tim Bliss</t>
+          <t>NA:TUS</t>
         </is>
       </c>
     </row>
@@ -5759,17 +5737,17 @@
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="C99" s="2" t="inlineStr">
+        <is>
           <t>15:00</t>
         </is>
       </c>
-      <c r="C99" s="2" t="inlineStr">
-        <is>
-          <t>16:30</t>
-        </is>
-      </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>Alicia Hahn</t>
+          <t>Tim Bliss</t>
         </is>
       </c>
     </row>
@@ -5781,17 +5759,17 @@
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
           <t>16:30</t>
         </is>
       </c>
-      <c r="C100" s="2" t="inlineStr">
-        <is>
-          <t>18:00</t>
-        </is>
-      </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>Yet More</t>
+          <t>Alicia Hahn</t>
         </is>
       </c>
     </row>
@@ -5803,17 +5781,17 @@
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="C101" s="2" t="inlineStr">
+        <is>
           <t>18:00</t>
         </is>
       </c>
-      <c r="C101" s="2" t="inlineStr">
-        <is>
-          <t>19:30</t>
-        </is>
-      </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>Dyzen</t>
+          <t>Yet More</t>
         </is>
       </c>
     </row>
@@ -5825,17 +5803,17 @@
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
           <t>19:30</t>
         </is>
       </c>
-      <c r="C102" s="2" t="inlineStr">
-        <is>
-          <t>21:00</t>
-        </is>
-      </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>Yulia Niko</t>
+          <t>Dyzen</t>
         </is>
       </c>
     </row>
@@ -5847,17 +5825,17 @@
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="C103" s="2" t="inlineStr">
+        <is>
           <t>21:00</t>
         </is>
       </c>
-      <c r="C103" s="2" t="inlineStr">
-        <is>
-          <t>22:30</t>
-        </is>
-      </c>
       <c r="D103" s="2" t="inlineStr">
         <is>
-          <t>Colyn b2b Sainte Vie</t>
+          <t>Yulia Niko</t>
         </is>
       </c>
     </row>
@@ -5869,39 +5847,39 @@
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="C104" s="2" t="inlineStr">
+        <is>
           <t>22:30</t>
         </is>
       </c>
-      <c r="C104" s="2" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>Chris Avantgarde b2b Konstantin Sibold</t>
+          <t>Colyn b2b Sainte Vie</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>THE GREAT LIBRARY</t>
+          <t>PLANAXIS</t>
         </is>
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>22:30</t>
         </is>
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
         <is>
-          <t>Radio Cargo</t>
+          <t>Chris Avantgarde b2b Konstantin Sibold</t>
         </is>
       </c>
     </row>
@@ -5913,17 +5891,17 @@
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="C106" s="2" t="inlineStr">
+        <is>
           <t>14:00</t>
         </is>
       </c>
-      <c r="C106" s="2" t="inlineStr">
-        <is>
-          <t>15:00</t>
-        </is>
-      </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>me n ü</t>
+          <t>Radio Cargo</t>
         </is>
       </c>
     </row>
@@ -5935,17 +5913,17 @@
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="C107" s="2" t="inlineStr">
+        <is>
           <t>15:00</t>
         </is>
       </c>
-      <c r="C107" s="2" t="inlineStr">
-        <is>
-          <t>16:00</t>
-        </is>
-      </c>
       <c r="D107" s="2" t="inlineStr">
         <is>
-          <t>Mesto</t>
+          <t>me n ü</t>
         </is>
       </c>
     </row>
@@ -5957,17 +5935,17 @@
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
           <t>16:00</t>
         </is>
       </c>
-      <c r="C108" s="2" t="inlineStr">
-        <is>
-          <t>17:00</t>
-        </is>
-      </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
-          <t>ZHU</t>
+          <t>Mesto</t>
         </is>
       </c>
     </row>
@@ -5979,17 +5957,17 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
           <t>17:00</t>
         </is>
       </c>
-      <c r="C109" s="2" t="inlineStr">
-        <is>
-          <t>18:00</t>
-        </is>
-      </c>
       <c r="D109" s="2" t="inlineStr">
         <is>
-          <t>Henri PFR</t>
+          <t>ZHU</t>
         </is>
       </c>
     </row>
@@ -6001,17 +5979,17 @@
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
           <t>18:00</t>
         </is>
       </c>
-      <c r="C110" s="2" t="inlineStr">
-        <is>
-          <t>19:00</t>
-        </is>
-      </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
-          <t>Chris Lorenzo</t>
+          <t>Henri PFR</t>
         </is>
       </c>
     </row>
@@ -6023,17 +6001,17 @@
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="C111" s="2" t="inlineStr">
+        <is>
           <t>19:00</t>
         </is>
       </c>
-      <c r="C111" s="2" t="inlineStr">
-        <is>
-          <t>20:00</t>
-        </is>
-      </c>
       <c r="D111" s="2" t="inlineStr">
         <is>
-          <t>Wilkinson</t>
+          <t>Chris Lorenzo</t>
         </is>
       </c>
     </row>
@@ -6045,17 +6023,17 @@
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C112" s="2" t="inlineStr">
+        <is>
           <t>20:00</t>
         </is>
       </c>
-      <c r="C112" s="2" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
       <c r="D112" s="2" t="inlineStr">
         <is>
-          <t>Sonny Fodera</t>
+          <t>Wilkinson</t>
         </is>
       </c>
     </row>
@@ -6067,17 +6045,17 @@
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="C113" s="2" t="inlineStr">
+        <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="C113" s="2" t="inlineStr">
-        <is>
-          <t>22:45</t>
-        </is>
-      </c>
       <c r="D113" s="2" t="inlineStr">
         <is>
-          <t>Lost Frequencies</t>
+          <t>Sonny Fodera</t>
         </is>
       </c>
     </row>
@@ -6089,17 +6067,17 @@
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C114" s="2" t="inlineStr">
+        <is>
           <t>22:45</t>
         </is>
       </c>
-      <c r="C114" s="2" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
       <c r="D114" s="2" t="inlineStr">
         <is>
-          <t>Gorgon City</t>
+          <t>Lost Frequencies</t>
         </is>
       </c>
     </row>
@@ -6111,39 +6089,39 @@
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
+          <t>22:45</t>
+        </is>
+      </c>
+      <c r="C115" s="2" t="inlineStr">
+        <is>
           <t>00:00</t>
         </is>
       </c>
-      <c r="C115" s="2" t="inlineStr">
-        <is>
-          <t>00:55</t>
-        </is>
-      </c>
       <c r="D115" s="2" t="inlineStr">
         <is>
-          <t>Netsky</t>
+          <t>Gorgon City</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>THE RAVE CAVE</t>
+          <t>THE GREAT LIBRARY</t>
         </is>
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>00:55</t>
         </is>
       </c>
       <c r="D116" s="2" t="inlineStr">
         <is>
-          <t>Charleen Herzig</t>
+          <t>Netsky</t>
         </is>
       </c>
     </row>
@@ -6155,17 +6133,17 @@
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="C117" s="2" t="inlineStr">
+        <is>
           <t>14:30</t>
         </is>
       </c>
-      <c r="C117" s="2" t="inlineStr">
-        <is>
-          <t>16:00</t>
-        </is>
-      </c>
       <c r="D117" s="2" t="inlineStr">
         <is>
-          <t>Simon B</t>
+          <t>Charleen Herzig</t>
         </is>
       </c>
     </row>
@@ -6177,17 +6155,17 @@
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="C118" s="2" t="inlineStr">
+        <is>
           <t>16:00</t>
         </is>
       </c>
-      <c r="C118" s="2" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
       <c r="D118" s="2" t="inlineStr">
         <is>
-          <t>Pat Krimson</t>
+          <t>Simon B</t>
         </is>
       </c>
     </row>
@@ -6199,17 +6177,17 @@
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="C119" s="2" t="inlineStr">
+        <is>
           <t>17:30</t>
         </is>
       </c>
-      <c r="C119" s="2" t="inlineStr">
-        <is>
-          <t>19:00</t>
-        </is>
-      </c>
       <c r="D119" s="2" t="inlineStr">
         <is>
-          <t>Roma</t>
+          <t>Pat Krimson</t>
         </is>
       </c>
     </row>
@@ -6221,17 +6199,17 @@
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="C120" s="2" t="inlineStr">
+        <is>
           <t>19:00</t>
         </is>
       </c>
-      <c r="C120" s="2" t="inlineStr">
-        <is>
-          <t>20:30</t>
-        </is>
-      </c>
       <c r="D120" s="2" t="inlineStr">
         <is>
-          <t>Ben Malone</t>
+          <t>Roma</t>
         </is>
       </c>
     </row>
@@ -6243,17 +6221,17 @@
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C121" s="2" t="inlineStr">
+        <is>
           <t>20:30</t>
         </is>
       </c>
-      <c r="C121" s="2" t="inlineStr">
-        <is>
-          <t>22:00</t>
-        </is>
-      </c>
       <c r="D121" s="2" t="inlineStr">
         <is>
-          <t>Jorn Pricez</t>
+          <t>Ben Malone</t>
         </is>
       </c>
     </row>
@@ -6265,17 +6243,17 @@
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="C122" s="2" t="inlineStr">
+        <is>
           <t>22:00</t>
         </is>
       </c>
-      <c r="C122" s="2" t="inlineStr">
-        <is>
-          <t>23:00</t>
-        </is>
-      </c>
       <c r="D122" s="2" t="inlineStr">
         <is>
-          <t>Flowchief</t>
+          <t>Jorn Pricez</t>
         </is>
       </c>
     </row>
@@ -6287,39 +6265,39 @@
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="C123" s="2" t="inlineStr">
+        <is>
           <t>23:00</t>
         </is>
       </c>
-      <c r="C123" s="2" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
       <c r="D123" s="2" t="inlineStr">
         <is>
-          <t>Netherworld</t>
+          <t>Flowchief</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>THE ROSE GARDEN</t>
+          <t>THE RAVE CAVE</t>
         </is>
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="C124" s="2" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="D124" s="2" t="inlineStr">
         <is>
-          <t>Quincy</t>
+          <t>Netherworld</t>
         </is>
       </c>
     </row>
@@ -6331,17 +6309,17 @@
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="C125" s="2" t="inlineStr">
+        <is>
           <t>13:30</t>
         </is>
       </c>
-      <c r="C125" s="2" t="inlineStr">
-        <is>
-          <t>15:00</t>
-        </is>
-      </c>
       <c r="D125" s="2" t="inlineStr">
         <is>
-          <t>Danny Corten</t>
+          <t>Quincy</t>
         </is>
       </c>
     </row>
@@ -6353,17 +6331,17 @@
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="C126" s="2" t="inlineStr">
+        <is>
           <t>15:00</t>
         </is>
       </c>
-      <c r="C126" s="2" t="inlineStr">
-        <is>
-          <t>16:30</t>
-        </is>
-      </c>
       <c r="D126" s="2" t="inlineStr">
         <is>
-          <t>Maite Dedecker</t>
+          <t>Danny Corten</t>
         </is>
       </c>
     </row>
@@ -6375,17 +6353,17 @@
       </c>
       <c r="B127" s="2" t="inlineStr">
         <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="C127" s="2" t="inlineStr">
+        <is>
           <t>16:30</t>
         </is>
       </c>
-      <c r="C127" s="2" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
       <c r="D127" s="2" t="inlineStr">
         <is>
-          <t>Dimitri Cooman</t>
+          <t>Maite Dedecker</t>
         </is>
       </c>
     </row>
@@ -6397,17 +6375,17 @@
       </c>
       <c r="B128" s="2" t="inlineStr">
         <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="C128" s="2" t="inlineStr">
+        <is>
           <t>17:30</t>
         </is>
       </c>
-      <c r="C128" s="2" t="inlineStr">
-        <is>
-          <t>18:30</t>
-        </is>
-      </c>
       <c r="D128" s="2" t="inlineStr">
         <is>
-          <t>DJ Ghost</t>
+          <t>Dimitri Cooman</t>
         </is>
       </c>
     </row>
@@ -6419,17 +6397,17 @@
       </c>
       <c r="B129" s="2" t="inlineStr">
         <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="C129" s="2" t="inlineStr">
+        <is>
           <t>18:30</t>
         </is>
       </c>
-      <c r="C129" s="2" t="inlineStr">
-        <is>
-          <t>19:30</t>
-        </is>
-      </c>
       <c r="D129" s="2" t="inlineStr">
         <is>
-          <t>Franky Kloeck</t>
+          <t>DJ Ghost</t>
         </is>
       </c>
     </row>
@@ -6441,17 +6419,17 @@
       </c>
       <c r="B130" s="2" t="inlineStr">
         <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="C130" s="2" t="inlineStr">
+        <is>
           <t>19:30</t>
         </is>
       </c>
-      <c r="C130" s="2" t="inlineStr">
-        <is>
-          <t>20:30</t>
-        </is>
-      </c>
       <c r="D130" s="2" t="inlineStr">
         <is>
-          <t>Jamie Dill</t>
+          <t>Franky Kloeck</t>
         </is>
       </c>
     </row>
@@ -6463,17 +6441,17 @@
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="C131" s="2" t="inlineStr">
+        <is>
           <t>20:30</t>
         </is>
       </c>
-      <c r="C131" s="2" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
       <c r="D131" s="2" t="inlineStr">
         <is>
-          <t>Youri Parker</t>
+          <t>Jamie Dill</t>
         </is>
       </c>
     </row>
@@ -6485,17 +6463,17 @@
       </c>
       <c r="B132" s="2" t="inlineStr">
         <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="C132" s="2" t="inlineStr">
+        <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="C132" s="2" t="inlineStr">
-        <is>
-          <t>23:00</t>
-        </is>
-      </c>
       <c r="D132" s="2" t="inlineStr">
         <is>
-          <t>BountyHunter</t>
+          <t>Youri Parker</t>
         </is>
       </c>
     </row>
@@ -6507,15 +6485,37 @@
       </c>
       <c r="B133" s="2" t="inlineStr">
         <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C133" s="2" t="inlineStr">
+        <is>
           <t>23:00</t>
         </is>
       </c>
-      <c r="C133" s="2" t="inlineStr">
+      <c r="D133" s="2" t="inlineStr">
+        <is>
+          <t>BountyHunter</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="2" t="inlineStr">
+        <is>
+          <t>THE ROSE GARDEN</t>
+        </is>
+      </c>
+      <c r="B134" s="2" t="inlineStr">
+        <is>
+          <t>23:00</t>
+        </is>
+      </c>
+      <c r="C134" s="2" t="inlineStr">
         <is>
           <t>01:00</t>
         </is>
       </c>
-      <c r="D133" s="2" t="inlineStr">
+      <c r="D134" s="2" t="inlineStr">
         <is>
           <t>Cherry Moon Legends (&amp; Friends)</t>
         </is>
@@ -6532,7 +6532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D130"/>
+  <dimension ref="A1:D129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -8517,7 +8517,7 @@
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>More to be announced</t>
+          <t>Vassy</t>
         </is>
       </c>
     </row>
@@ -8529,17 +8529,17 @@
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>Vassy</t>
+          <t>Yves V b2b StadiumX</t>
         </is>
       </c>
     </row>
@@ -8551,17 +8551,17 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>Yves V b2b StadiumX</t>
+          <t>Sick individuals</t>
         </is>
       </c>
     </row>
@@ -8573,17 +8573,17 @@
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>Sick individuals</t>
+          <t>Deorro</t>
         </is>
       </c>
     </row>
@@ -8595,17 +8595,17 @@
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>Deorro</t>
+          <t>Laidback Luke</t>
         </is>
       </c>
     </row>
@@ -8617,17 +8617,17 @@
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>Laidback Luke</t>
+          <t>Superheroes</t>
         </is>
       </c>
     </row>
@@ -8639,17 +8639,17 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>Superheroes</t>
+          <t>Quintino</t>
         </is>
       </c>
     </row>
@@ -8661,39 +8661,39 @@
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>23:50</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>Quintino</t>
+          <t>Chuckie</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>PLANAXIS</t>
+          <t>THE GREAT LIBRARY</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>23:50</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>Chuckie</t>
+          <t>Zero Gravity</t>
         </is>
       </c>
     </row>
@@ -8705,17 +8705,17 @@
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>Zero Gravity</t>
+          <t>Lucca van Damme</t>
         </is>
       </c>
     </row>
@@ -8727,17 +8727,17 @@
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>Lucca van Damme</t>
+          <t>Diego Miranda b2b Jerry Davila</t>
         </is>
       </c>
     </row>
@@ -8749,17 +8749,17 @@
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>Diego Miranda b2b Jerry Davila</t>
+          <t>Darren Styles</t>
         </is>
       </c>
     </row>
@@ -8771,17 +8771,17 @@
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>Darren Styles</t>
+          <t>Kaaze</t>
         </is>
       </c>
     </row>
@@ -8793,17 +8793,17 @@
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="D103" s="2" t="inlineStr">
         <is>
-          <t>Kaaze</t>
+          <t>Paris Hilton</t>
         </is>
       </c>
     </row>
@@ -8815,17 +8815,17 @@
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>Paris Hilton</t>
+          <t>Joel Corry</t>
         </is>
       </c>
     </row>
@@ -8837,17 +8837,17 @@
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
         <is>
-          <t>Joel Corry</t>
+          <t>NERVO</t>
         </is>
       </c>
     </row>
@@ -8859,17 +8859,17 @@
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>NERVO</t>
+          <t>Nico Moreno</t>
         </is>
       </c>
     </row>
@@ -8881,17 +8881,17 @@
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr">
         <is>
-          <t>Nico Moreno</t>
+          <t>Bassjackers</t>
         </is>
       </c>
     </row>
@@ -8903,17 +8903,17 @@
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
-          <t>Bassjackers</t>
+          <t>Dimitri Vegas b2b Nico Moreno</t>
         </is>
       </c>
     </row>
@@ -8925,39 +8925,39 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>23:55</t>
         </is>
       </c>
       <c r="D109" s="2" t="inlineStr">
         <is>
-          <t>Dimitri Vegas b2b Nico Moreno</t>
+          <t>Brennan Heart</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>THE GREAT LIBRARY</t>
+          <t>THE RAVE CAVE</t>
         </is>
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>23:55</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
-          <t>Brennan Heart</t>
+          <t>Benny Plays</t>
         </is>
       </c>
     </row>
@@ -8969,17 +8969,17 @@
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="D111" s="2" t="inlineStr">
         <is>
-          <t>Benny Plays</t>
+          <t>EME</t>
         </is>
       </c>
     </row>
@@ -8991,17 +8991,17 @@
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="D112" s="2" t="inlineStr">
         <is>
-          <t>EME</t>
+          <t>Kriss Reeve</t>
         </is>
       </c>
     </row>
@@ -9013,17 +9013,17 @@
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="D113" s="2" t="inlineStr">
         <is>
-          <t>Kriss Reeve</t>
+          <t>Muze</t>
         </is>
       </c>
     </row>
@@ -9035,17 +9035,17 @@
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="D114" s="2" t="inlineStr">
         <is>
-          <t>Muze</t>
+          <t>Mr. Rewind</t>
         </is>
       </c>
     </row>
@@ -9057,17 +9057,17 @@
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="C115" s="2" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="D115" s="2" t="inlineStr">
         <is>
-          <t>Mr. Rewind</t>
+          <t>D. Guaetta b2b Neon</t>
         </is>
       </c>
     </row>
@@ -9079,17 +9079,17 @@
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="D116" s="2" t="inlineStr">
         <is>
-          <t>D. Guaetta b2b Neon</t>
+          <t>Hyalyte</t>
         </is>
       </c>
     </row>
@@ -9101,17 +9101,17 @@
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="D117" s="2" t="inlineStr">
         <is>
-          <t>Hyalyte</t>
+          <t>Leenders</t>
         </is>
       </c>
     </row>
@@ -9123,39 +9123,39 @@
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="D118" s="2" t="inlineStr">
         <is>
-          <t>Leenders</t>
+          <t>DXNØ</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>THE RAVE CAVE</t>
+          <t>THE ROSE GARDEN</t>
         </is>
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="C119" s="2" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="D119" s="2" t="inlineStr">
         <is>
-          <t>DXNØ</t>
+          <t>BassBrain</t>
         </is>
       </c>
     </row>
@@ -9167,17 +9167,17 @@
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="D120" s="2" t="inlineStr">
         <is>
-          <t>BassBrain</t>
+          <t>Lost Identity</t>
         </is>
       </c>
     </row>
@@ -9189,17 +9189,17 @@
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="C121" s="2" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="D121" s="2" t="inlineStr">
         <is>
-          <t>Lost Identity</t>
+          <t>D-Charged b2b Serzo</t>
         </is>
       </c>
     </row>
@@ -9211,17 +9211,17 @@
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="C122" s="2" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="D122" s="2" t="inlineStr">
         <is>
-          <t>D-Charged b2b Serzo</t>
+          <t>Mark With A K &amp; MC Chucky</t>
         </is>
       </c>
     </row>
@@ -9233,17 +9233,17 @@
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="C123" s="2" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="D123" s="2" t="inlineStr">
         <is>
-          <t>Mark With A K &amp; MC Chucky</t>
+          <t>Hard Driver</t>
         </is>
       </c>
     </row>
@@ -9255,17 +9255,17 @@
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C124" s="2" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="D124" s="2" t="inlineStr">
         <is>
-          <t>Hard Driver</t>
+          <t>The Purge</t>
         </is>
       </c>
     </row>
@@ -9277,17 +9277,17 @@
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="C125" s="2" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="D125" s="2" t="inlineStr">
         <is>
-          <t>The Purge</t>
+          <t>Sound Rush</t>
         </is>
       </c>
     </row>
@@ -9299,17 +9299,17 @@
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="C126" s="2" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="D126" s="2" t="inlineStr">
         <is>
-          <t>Sound Rush</t>
+          <t>Coone</t>
         </is>
       </c>
     </row>
@@ -9321,17 +9321,17 @@
       </c>
       <c r="B127" s="2" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="C127" s="2" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="D127" s="2" t="inlineStr">
         <is>
-          <t>Coone</t>
+          <t>Da Tweekaz</t>
         </is>
       </c>
     </row>
@@ -9343,17 +9343,17 @@
       </c>
       <c r="B128" s="2" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="C128" s="2" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>22:15</t>
         </is>
       </c>
       <c r="D128" s="2" t="inlineStr">
         <is>
-          <t>Da Tweekaz</t>
+          <t>Warface</t>
         </is>
       </c>
     </row>
@@ -9365,37 +9365,15 @@
       </c>
       <c r="B129" s="2" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>22:15</t>
         </is>
       </c>
       <c r="C129" s="2" t="inlineStr">
         <is>
-          <t>22:15</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="D129" s="2" t="inlineStr">
-        <is>
-          <t>Warface</t>
-        </is>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" s="2" t="inlineStr">
-        <is>
-          <t>THE ROSE GARDEN</t>
-        </is>
-      </c>
-      <c r="B130" s="2" t="inlineStr">
-        <is>
-          <t>22:15</t>
-        </is>
-      </c>
-      <c r="C130" s="2" t="inlineStr">
-        <is>
-          <t>23:00</t>
-        </is>
-      </c>
-      <c r="D130" s="2" t="inlineStr">
         <is>
           <t>The Straikerz</t>
         </is>

</xml_diff>